<commit_message>
DONALD-2 Correction of the variables according to today's discussion. Only the operation for education and the variable for dietary assessment are missing.
</commit_message>
<xml_diff>
--- a/rmonize/data_dictionary/DD_DONALD_P1.xlsx
+++ b/rmonize/data_dictionary/DD_DONALD_P1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="282">
   <si>
     <t>index</t>
   </si>
@@ -49,9 +49,6 @@
     <t>sex</t>
   </si>
   <si>
-    <t>EDU_LEVEL_P</t>
-  </si>
-  <si>
     <t>TOT_PA_QX</t>
   </si>
   <si>
@@ -781,9 +778,6 @@
     <t>Physical activity from questionnaire data [MET-hr/week]</t>
   </si>
   <si>
-    <t>parental education status</t>
-  </si>
-  <si>
     <t>Age [years] at dietary assessment (1. record day)</t>
   </si>
   <si>
@@ -796,36 +790,6 @@
     <t>integer</t>
   </si>
   <si>
-    <t>Early Childhood Education</t>
-  </si>
-  <si>
-    <t>Primary Education</t>
-  </si>
-  <si>
-    <t>Lower Secondary Education</t>
-  </si>
-  <si>
-    <t>Upper Secondary Education</t>
-  </si>
-  <si>
-    <t>Post-secondary non-tertiary education</t>
-  </si>
-  <si>
-    <t>Short-Cycle Tertiary Education</t>
-  </si>
-  <si>
-    <t>Bachelor's or equivalent level</t>
-  </si>
-  <si>
-    <t>Master's or equivalent level</t>
-  </si>
-  <si>
-    <t>Doctoral or equivalent level</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
     <t>Smoker in Household [yes/no]</t>
   </si>
   <si>
@@ -836,6 +800,72 @@
   </si>
   <si>
     <t>Geschlecht</t>
+  </si>
+  <si>
+    <t>m_schulab</t>
+  </si>
+  <si>
+    <t>v_schulab</t>
+  </si>
+  <si>
+    <t>b_berufsab</t>
+  </si>
+  <si>
+    <t>v_berufsab</t>
+  </si>
+  <si>
+    <t>Schuldbildung der Mutter</t>
+  </si>
+  <si>
+    <t>Schuldbildung des Vaters</t>
+  </si>
+  <si>
+    <t>Berufsabschluss der Mutter</t>
+  </si>
+  <si>
+    <t>Berufsabschluss des Vaters</t>
+  </si>
+  <si>
+    <t>Volks-/Hauptschulabschluss</t>
+  </si>
+  <si>
+    <t>Mittlere Reife, Realschulabschluss (Fachschulreife)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fachhochschulreife, Abschluss einer Fachoberschule etc.       </t>
+  </si>
+  <si>
+    <t>Abitur (Hochschulreife)</t>
+  </si>
+  <si>
+    <t>keinen dieser Abschlüsse</t>
+  </si>
+  <si>
+    <t>m_berufsab</t>
+  </si>
+  <si>
+    <t>Lehre (beruflich-betriebliche Ausbildung)</t>
+  </si>
+  <si>
+    <t>Berufsschule, Handelsschule (berufl.-schulische Ausbildung)</t>
+  </si>
+  <si>
+    <t>Fachschule (z.B. Meister-Technikerschule, Berufs/Fachakademie)</t>
+  </si>
+  <si>
+    <t>Fachhochschule, Ingenieurschule</t>
+  </si>
+  <si>
+    <t>Universität, Hochschule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">anderer Abschluss (bis 3/2016 berufl. Praktikum)                          </t>
+  </si>
+  <si>
+    <t xml:space="preserve">kein beruflicher Abschluss     </t>
+  </si>
+  <si>
+    <t>noch in beruflicher Ausbildung (Auszubildener / Student)</t>
   </si>
 </sst>
 </file>
@@ -1174,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D130"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="22.54296875" customWidth="1"/>
@@ -1207,7 +1237,7 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1218,10 +1248,10 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="D3" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1232,7 +1262,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
@@ -1243,13 +1273,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>9</v>
+        <v>260</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="D5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -1257,13 +1287,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>10</v>
+        <v>261</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
       <c r="D6" t="s">
-        <v>5</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -1271,13 +1301,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>11</v>
+        <v>262</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D7" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -1285,13 +1315,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>12</v>
+        <v>263</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>132</v>
+        <v>267</v>
       </c>
       <c r="D8" t="s">
-        <v>5</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -1299,10 +1329,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>133</v>
+        <v>251</v>
       </c>
       <c r="D9" t="s">
         <v>5</v>
@@ -1313,13 +1343,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>134</v>
+        <v>256</v>
       </c>
       <c r="D10" t="s">
-        <v>5</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -1327,10 +1357,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
@@ -1341,10 +1371,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D12" t="s">
         <v>5</v>
@@ -1355,10 +1385,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D13" t="s">
         <v>5</v>
@@ -1369,10 +1399,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
@@ -1383,10 +1413,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
@@ -1397,10 +1427,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D16" t="s">
         <v>5</v>
@@ -1411,10 +1441,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D17" t="s">
         <v>5</v>
@@ -1425,10 +1455,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D18" t="s">
         <v>5</v>
@@ -1439,10 +1469,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D19" t="s">
         <v>5</v>
@@ -1453,10 +1483,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D20" t="s">
         <v>5</v>
@@ -1467,10 +1497,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D21" t="s">
         <v>5</v>
@@ -1481,10 +1511,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D22" t="s">
         <v>5</v>
@@ -1495,10 +1525,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D23" t="s">
         <v>5</v>
@@ -1509,10 +1539,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D24" t="s">
         <v>5</v>
@@ -1523,10 +1553,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D25" t="s">
         <v>5</v>
@@ -1537,10 +1567,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D26" t="s">
         <v>5</v>
@@ -1551,10 +1581,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D27" t="s">
         <v>5</v>
@@ -1565,10 +1595,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D28" t="s">
         <v>5</v>
@@ -1579,10 +1609,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D29" t="s">
         <v>5</v>
@@ -1593,10 +1623,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D30" t="s">
         <v>5</v>
@@ -1607,10 +1637,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D31" t="s">
         <v>5</v>
@@ -1621,10 +1651,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D32" t="s">
         <v>5</v>
@@ -1635,10 +1665,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D33" t="s">
         <v>5</v>
@@ -1649,10 +1679,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D34" t="s">
         <v>5</v>
@@ -1663,10 +1693,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="D35" t="s">
         <v>5</v>
@@ -1677,10 +1707,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D36" t="s">
         <v>5</v>
@@ -1691,10 +1721,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="D37" t="s">
         <v>5</v>
@@ -1705,10 +1735,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="D38" t="s">
         <v>5</v>
@@ -1719,10 +1749,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D39" t="s">
         <v>5</v>
@@ -1733,10 +1763,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D40" t="s">
         <v>5</v>
@@ -1747,10 +1777,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D41" t="s">
         <v>5</v>
@@ -1761,10 +1791,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D42" t="s">
         <v>5</v>
@@ -1775,10 +1805,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D43" t="s">
         <v>5</v>
@@ -1789,10 +1819,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D44" t="s">
         <v>5</v>
@@ -1803,10 +1833,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D45" t="s">
         <v>5</v>
@@ -1817,10 +1847,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D46" t="s">
         <v>5</v>
@@ -1831,10 +1861,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D47" t="s">
         <v>5</v>
@@ -1845,10 +1875,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D48" t="s">
         <v>5</v>
@@ -1859,10 +1889,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D49" t="s">
         <v>5</v>
@@ -1873,10 +1903,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D50" t="s">
         <v>5</v>
@@ -1887,10 +1917,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D51" t="s">
         <v>5</v>
@@ -1901,10 +1931,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D52" t="s">
         <v>5</v>
@@ -1915,10 +1945,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D53" t="s">
         <v>5</v>
@@ -1929,10 +1959,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D54" t="s">
         <v>5</v>
@@ -1943,10 +1973,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D55" t="s">
         <v>5</v>
@@ -1957,10 +1987,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D56" t="s">
         <v>5</v>
@@ -1971,10 +2001,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D57" t="s">
         <v>5</v>
@@ -1985,10 +2015,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D58" t="s">
         <v>5</v>
@@ -1999,10 +2029,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D59" t="s">
         <v>5</v>
@@ -2013,10 +2043,10 @@
         <v>59</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D60" t="s">
         <v>5</v>
@@ -2027,10 +2057,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D61" t="s">
         <v>5</v>
@@ -2041,10 +2071,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D62" t="s">
         <v>5</v>
@@ -2055,10 +2085,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D63" t="s">
         <v>5</v>
@@ -2069,10 +2099,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D64" t="s">
         <v>5</v>
@@ -2083,10 +2113,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D65" t="s">
         <v>5</v>
@@ -2097,10 +2127,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D66" t="s">
         <v>5</v>
@@ -2111,10 +2141,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D67" t="s">
         <v>5</v>
@@ -2125,10 +2155,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D68" t="s">
         <v>5</v>
@@ -2139,10 +2169,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D69" t="s">
         <v>5</v>
@@ -2153,10 +2183,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D70" t="s">
         <v>5</v>
@@ -2167,10 +2197,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="D71" t="s">
         <v>5</v>
@@ -2181,10 +2211,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D72" t="s">
         <v>5</v>
@@ -2195,10 +2225,10 @@
         <v>72</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D73" t="s">
         <v>5</v>
@@ -2209,10 +2239,10 @@
         <v>73</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="D74" t="s">
         <v>5</v>
@@ -2223,10 +2253,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D75" t="s">
         <v>5</v>
@@ -2237,10 +2267,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D76" t="s">
         <v>5</v>
@@ -2251,10 +2281,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D77" t="s">
         <v>5</v>
@@ -2265,10 +2295,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D78" t="s">
         <v>5</v>
@@ -2279,10 +2309,10 @@
         <v>78</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D79" t="s">
         <v>5</v>
@@ -2293,10 +2323,10 @@
         <v>79</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D80" t="s">
         <v>5</v>
@@ -2307,10 +2337,10 @@
         <v>80</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D81" t="s">
         <v>5</v>
@@ -2321,10 +2351,10 @@
         <v>81</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D82" t="s">
         <v>5</v>
@@ -2335,10 +2365,10 @@
         <v>82</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D83" t="s">
         <v>5</v>
@@ -2349,10 +2379,10 @@
         <v>83</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="D84" t="s">
         <v>5</v>
@@ -2363,10 +2393,10 @@
         <v>84</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D85" t="s">
         <v>5</v>
@@ -2377,10 +2407,10 @@
         <v>85</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="D86" t="s">
         <v>5</v>
@@ -2391,10 +2421,10 @@
         <v>86</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="D87" t="s">
         <v>5</v>
@@ -2405,10 +2435,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D88" t="s">
         <v>5</v>
@@ -2419,10 +2449,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="D89" t="s">
         <v>5</v>
@@ -2433,10 +2463,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="D90" t="s">
         <v>5</v>
@@ -2447,10 +2477,10 @@
         <v>90</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="D91" t="s">
         <v>5</v>
@@ -2461,10 +2491,10 @@
         <v>91</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D92" t="s">
         <v>5</v>
@@ -2475,10 +2505,10 @@
         <v>92</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D93" t="s">
         <v>5</v>
@@ -2489,10 +2519,10 @@
         <v>93</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D94" t="s">
         <v>5</v>
@@ -2503,10 +2533,10 @@
         <v>94</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D95" t="s">
         <v>5</v>
@@ -2517,10 +2547,10 @@
         <v>95</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D96" t="s">
         <v>5</v>
@@ -2531,10 +2561,10 @@
         <v>96</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="D97" t="s">
         <v>5</v>
@@ -2545,10 +2575,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="D98" t="s">
         <v>5</v>
@@ -2559,10 +2589,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="D99" t="s">
         <v>5</v>
@@ -2573,10 +2603,10 @@
         <v>99</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D100" t="s">
         <v>5</v>
@@ -2587,10 +2617,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="D101" t="s">
         <v>5</v>
@@ -2601,10 +2631,10 @@
         <v>101</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="D102" t="s">
         <v>5</v>
@@ -2615,10 +2645,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D103" t="s">
         <v>5</v>
@@ -2629,10 +2659,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="D104" t="s">
         <v>5</v>
@@ -2643,10 +2673,10 @@
         <v>104</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="D105" t="s">
         <v>5</v>
@@ -2657,10 +2687,10 @@
         <v>105</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="D106" t="s">
         <v>5</v>
@@ -2671,10 +2701,10 @@
         <v>106</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D107" t="s">
         <v>5</v>
@@ -2685,10 +2715,10 @@
         <v>107</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="D108" t="s">
         <v>5</v>
@@ -2699,10 +2729,10 @@
         <v>108</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="D109" t="s">
         <v>5</v>
@@ -2713,10 +2743,10 @@
         <v>109</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="D110" t="s">
         <v>5</v>
@@ -2727,10 +2757,10 @@
         <v>110</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="D111" t="s">
         <v>5</v>
@@ -2741,10 +2771,10 @@
         <v>111</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="D112" t="s">
         <v>5</v>
@@ -2755,10 +2785,10 @@
         <v>112</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="D113" t="s">
         <v>5</v>
@@ -2769,10 +2799,10 @@
         <v>113</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="D114" t="s">
         <v>5</v>
@@ -2783,10 +2813,10 @@
         <v>114</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="D115" t="s">
         <v>5</v>
@@ -2797,10 +2827,10 @@
         <v>115</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="D116" t="s">
         <v>5</v>
@@ -2811,10 +2841,10 @@
         <v>116</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D117" t="s">
         <v>5</v>
@@ -2825,10 +2855,10 @@
         <v>117</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="D118" t="s">
         <v>5</v>
@@ -2839,10 +2869,10 @@
         <v>118</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D119" t="s">
         <v>5</v>
@@ -2853,10 +2883,10 @@
         <v>119</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="D120" t="s">
         <v>5</v>
@@ -2867,10 +2897,10 @@
         <v>120</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="D121" t="s">
         <v>5</v>
@@ -2881,10 +2911,10 @@
         <v>121</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D122" t="s">
         <v>5</v>
@@ -2895,10 +2925,10 @@
         <v>122</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="D123" t="s">
         <v>5</v>
@@ -2909,10 +2939,10 @@
         <v>123</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="D124" t="s">
         <v>5</v>
@@ -2923,10 +2953,10 @@
         <v>124</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="D125" t="s">
         <v>5</v>
@@ -2937,10 +2967,10 @@
         <v>125</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="D126" t="s">
         <v>5</v>
@@ -2951,12 +2981,54 @@
         <v>126</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D127" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="D128" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D129" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="D130" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2968,7 +3040,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2994,7 +3066,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -3005,139 +3077,315 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>9</v>
+        <v>260</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>9</v>
+        <v>260</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>9</v>
+        <v>260</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>9</v>
+        <v>260</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>9</v>
+        <v>260</v>
       </c>
       <c r="B8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>9</v>
+        <v>261</v>
       </c>
       <c r="B9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>9</v>
+        <v>261</v>
       </c>
       <c r="B10">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C10" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>9</v>
+        <v>261</v>
       </c>
       <c r="B11">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C11" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>9</v>
+        <v>261</v>
       </c>
       <c r="B12">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>9</v>
+        <v>261</v>
       </c>
       <c r="B13">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>11</v>
+        <v>273</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>11</v>
+        <v>273</v>
       </c>
       <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B17">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B18">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B19">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B20">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B21">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B22">
         <v>1</v>
       </c>
-      <c r="C15" t="s">
-        <v>270</v>
+      <c r="C22" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B23">
+        <v>2</v>
+      </c>
+      <c r="C23" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B24">
+        <v>3</v>
+      </c>
+      <c r="C24" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B25">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B26">
+        <v>5</v>
+      </c>
+      <c r="C26" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B27">
+        <v>6</v>
+      </c>
+      <c r="C27" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B28">
+        <v>7</v>
+      </c>
+      <c r="C28" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B29">
+        <v>8</v>
+      </c>
+      <c r="C29" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B30">
+        <v>0</v>
+      </c>
+      <c r="C30" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
+        <v>258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DONALD-4 all files for P1 and P2
</commit_message>
<xml_diff>
--- a/rmonize/data_dictionary/DD_DONALD_P1.xlsx
+++ b/rmonize/data_dictionary/DD_DONALD_P1.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E2CDD8-DCB9-4A5F-866A-B5B1214CAEFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14895" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="281">
   <si>
     <t>index</t>
   </si>
@@ -808,12 +809,6 @@
     <t>v_schulab</t>
   </si>
   <si>
-    <t>b_berufsab</t>
-  </si>
-  <si>
-    <t>v_berufsab</t>
-  </si>
-  <si>
     <t>Schuldbildung der Mutter</t>
   </si>
   <si>
@@ -841,9 +836,6 @@
     <t>keinen dieser Abschlüsse</t>
   </si>
   <si>
-    <t>m_berufsab</t>
-  </si>
-  <si>
     <t>Lehre (beruflich-betriebliche Ausbildung)</t>
   </si>
   <si>
@@ -866,12 +858,18 @@
   </si>
   <si>
     <t>noch in beruflicher Ausbildung (Auszubildener / Student)</t>
+  </si>
+  <si>
+    <t>m_berufab</t>
+  </si>
+  <si>
+    <t>v_berufab</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -926,7 +924,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1203,16 +1201,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D130"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.54296875" customWidth="1"/>
-    <col min="3" max="3" width="55.26953125" customWidth="1"/>
-    <col min="4" max="4" width="25.81640625" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" customWidth="1"/>
+    <col min="3" max="3" width="55.28515625" customWidth="1"/>
+    <col min="4" max="4" width="25.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1226,7 +1224,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1240,7 +1238,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1254,7 +1252,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1268,7 +1266,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1276,13 +1274,13 @@
         <v>260</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D5" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1290,41 +1288,41 @@
         <v>261</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D6" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>262</v>
+        <v>279</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D7" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D8" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1338,7 +1336,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1352,7 +1350,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1366,7 +1364,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1380,7 +1378,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1394,7 +1392,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1408,7 +1406,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1422,7 +1420,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1436,7 +1434,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1450,7 +1448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1464,7 +1462,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1478,7 +1476,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1492,7 +1490,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1506,7 +1504,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1520,7 +1518,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1534,7 +1532,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1548,7 +1546,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1562,7 +1560,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1576,7 +1574,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1590,7 +1588,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1604,7 +1602,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1618,7 +1616,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1632,7 +1630,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1646,7 +1644,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1660,7 +1658,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1674,7 +1672,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1688,7 +1686,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1702,7 +1700,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1716,7 +1714,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1730,7 +1728,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1744,7 +1742,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1758,7 +1756,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1772,7 +1770,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1786,7 +1784,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1800,7 +1798,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1814,7 +1812,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1828,7 +1826,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1842,7 +1840,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1856,7 +1854,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1870,7 +1868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1884,7 +1882,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1898,7 +1896,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1912,7 +1910,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1926,7 +1924,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1940,7 +1938,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1954,7 +1952,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1968,7 +1966,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1982,7 +1980,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1996,7 +1994,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2010,7 +2008,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2024,7 +2022,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2038,7 +2036,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2052,7 +2050,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2066,7 +2064,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2080,7 +2078,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2094,7 +2092,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2108,7 +2106,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2122,7 +2120,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2136,7 +2134,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2150,7 +2148,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2164,7 +2162,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2178,7 +2176,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2192,7 +2190,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2206,7 +2204,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2220,7 +2218,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2234,7 +2232,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2248,7 +2246,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2262,7 +2260,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2276,7 +2274,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2290,7 +2288,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2304,7 +2302,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2318,7 +2316,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2332,7 +2330,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2346,7 +2344,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2360,7 +2358,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2374,7 +2372,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2388,7 +2386,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2402,7 +2400,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2416,7 +2414,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2430,7 +2428,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2444,7 +2442,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2458,7 +2456,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2472,7 +2470,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2486,7 +2484,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2500,7 +2498,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2514,7 +2512,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2528,7 +2526,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -2542,7 +2540,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -2556,7 +2554,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -2570,7 +2568,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -2584,7 +2582,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -2598,7 +2596,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -2612,7 +2610,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -2626,7 +2624,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -2640,7 +2638,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -2654,7 +2652,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -2668,7 +2666,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -2682,7 +2680,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -2696,7 +2694,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -2710,7 +2708,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -2724,7 +2722,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -2738,7 +2736,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -2752,7 +2750,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -2766,7 +2764,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -2780,7 +2778,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -2794,7 +2792,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
@@ -2808,7 +2806,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -2822,7 +2820,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -2836,7 +2834,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
@@ -2850,7 +2848,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
@@ -2864,7 +2862,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
@@ -2878,7 +2876,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -2892,7 +2890,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -2906,7 +2904,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -2920,7 +2918,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>122</v>
       </c>
@@ -2934,7 +2932,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>123</v>
       </c>
@@ -2948,7 +2946,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>124</v>
       </c>
@@ -2962,7 +2960,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>125</v>
       </c>
@@ -2976,7 +2974,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>126</v>
       </c>
@@ -2990,7 +2988,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>127</v>
       </c>
@@ -3004,7 +3002,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>128</v>
       </c>
@@ -3018,7 +3016,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>129</v>
       </c>
@@ -3039,15 +3037,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="19.36328125" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -3058,7 +3056,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -3069,7 +3067,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -3080,7 +3078,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>260</v>
       </c>
@@ -3088,10 +3086,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>260</v>
       </c>
@@ -3099,10 +3097,10 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>260</v>
       </c>
@@ -3110,10 +3108,10 @@
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>260</v>
       </c>
@@ -3121,10 +3119,10 @@
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>260</v>
       </c>
@@ -3132,10 +3130,10 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>261</v>
       </c>
@@ -3143,10 +3141,10 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>261</v>
       </c>
@@ -3154,10 +3152,10 @@
         <v>2</v>
       </c>
       <c r="C10" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>261</v>
       </c>
@@ -3165,10 +3163,10 @@
         <v>3</v>
       </c>
       <c r="C11" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>261</v>
       </c>
@@ -3176,10 +3174,10 @@
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>261</v>
       </c>
@@ -3187,186 +3185,186 @@
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="B16">
         <v>3</v>
       </c>
       <c r="C16" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="B17">
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="B18">
         <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="B19">
         <v>6</v>
       </c>
       <c r="C19" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>279</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
-        <v>273</v>
       </c>
       <c r="B20">
         <v>7</v>
       </c>
       <c r="C20" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="B21">
         <v>8</v>
       </c>
       <c r="C21" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="B23">
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="B24">
         <v>3</v>
       </c>
       <c r="C24" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="B25">
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="B26">
         <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="B27">
         <v>6</v>
       </c>
       <c r="C27" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="B28">
         <v>7</v>
       </c>
       <c r="C28" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>280</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29" s="3" t="s">
-        <v>263</v>
       </c>
       <c r="B29">
         <v>8</v>
       </c>
       <c r="C29" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>10</v>
       </c>
@@ -3377,7 +3375,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>10</v>
       </c>

</xml_diff>